<commit_message>
128, 256 pt result 저장
</commit_message>
<xml_diff>
--- a/연구코드/data/강남/aec/강남_z_bounds.xlsx
+++ b/연구코드/data/강남/aec/강남_z_bounds.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="12">
   <si>
     <t>No</t>
   </si>
@@ -50,12 +50,6 @@
   </si>
   <si>
     <t>t12_missing</t>
-  </si>
-  <si>
-    <t>hip_missing</t>
-  </si>
-  <si>
-    <t>nifti_fail</t>
   </si>
 </sst>
 </file>
@@ -38248,28 +38242,28 @@
         <v>6740540</v>
       </c>
       <c r="C1183">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D1183">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="E1183">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="F1183">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G1183">
-        <v>194</v>
+        <v>355</v>
       </c>
       <c r="H1183">
-        <v>383.4</v>
+        <v>428.5</v>
       </c>
       <c r="I1183">
-        <v>577.4</v>
+        <v>73.5</v>
       </c>
       <c r="J1183" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1184" spans="1:10">
@@ -39115,22 +39109,22 @@
         <v>199</v>
       </c>
       <c r="D1210">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E1210">
         <v>1</v>
       </c>
       <c r="F1210">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G1210">
-        <v>455</v>
+        <v>457.5</v>
       </c>
       <c r="H1210">
         <v>-4.282</v>
       </c>
       <c r="I1210">
-        <v>-459.282</v>
+        <v>-461.782</v>
       </c>
       <c r="J1210" t="s">
         <v>11</v>
@@ -43563,22 +43557,22 @@
         <v>160</v>
       </c>
       <c r="D1349">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E1349">
         <v>1</v>
       </c>
       <c r="F1349">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="G1349">
-        <v>382.5</v>
+        <v>372.5</v>
       </c>
       <c r="H1349">
         <v>22.294</v>
       </c>
       <c r="I1349">
-        <v>-360.207</v>
+        <v>-350.207</v>
       </c>
       <c r="J1349" t="s">
         <v>11</v>
@@ -53771,25 +53765,25 @@
         <v>118</v>
       </c>
       <c r="D1668">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E1668">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="F1668">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="G1668">
-        <v>168</v>
+        <v>360</v>
       </c>
       <c r="H1668">
-        <v>438.4</v>
+        <v>487.5</v>
       </c>
       <c r="I1668">
-        <v>606.4</v>
+        <v>127.5</v>
       </c>
       <c r="J1668" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1669" spans="1:10">
@@ -60264,28 +60258,28 @@
         <v>9715511</v>
       </c>
       <c r="C1871">
-        <v>98</v>
+        <v>144</v>
       </c>
       <c r="D1871">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="E1871">
-        <v>98</v>
+        <v>15</v>
       </c>
       <c r="F1871">
-        <v>1</v>
+        <v>137</v>
       </c>
       <c r="G1871">
-        <v>291</v>
+        <v>366</v>
       </c>
       <c r="H1871">
-        <v>1691</v>
+        <v>1741.8</v>
       </c>
       <c r="I1871">
-        <v>1982</v>
+        <v>1375.8</v>
       </c>
       <c r="J1871" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1872" spans="1:10">
@@ -64776,28 +64770,28 @@
         <v>9930443</v>
       </c>
       <c r="C2012">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D2012">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="E2012">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="F2012">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="G2012">
-        <v>168.75</v>
+        <v>380</v>
       </c>
       <c r="H2012">
-        <v>-129</v>
+        <v>-132.75</v>
       </c>
       <c r="I2012">
-        <v>-297.75</v>
+        <v>-512.75</v>
       </c>
       <c r="J2012" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2013" spans="1:10">
@@ -64968,28 +64962,28 @@
         <v>9944576</v>
       </c>
       <c r="C2018">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D2018">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="E2018">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="F2018">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G2018">
-        <v>148</v>
+        <v>384</v>
       </c>
       <c r="H2018">
         <v>1693</v>
       </c>
       <c r="I2018">
-        <v>1545</v>
+        <v>1309</v>
       </c>
       <c r="J2018" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2019" spans="1:10">
@@ -65767,8 +65761,29 @@
       <c r="B2043">
         <v>9995235</v>
       </c>
+      <c r="C2043">
+        <v>203</v>
+      </c>
+      <c r="D2043">
+        <v>137</v>
+      </c>
+      <c r="E2043">
+        <v>53</v>
+      </c>
+      <c r="F2043">
+        <v>189</v>
+      </c>
+      <c r="G2043">
+        <v>340</v>
+      </c>
+      <c r="H2043">
+        <v>-116.467</v>
+      </c>
+      <c r="I2043">
+        <v>-456.467</v>
+      </c>
       <c r="J2043" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2044" spans="1:10">

</xml_diff>